<commit_message>
fix:resolve issue with buy API call
</commit_message>
<xml_diff>
--- a/src/allocations.xlsx
+++ b/src/allocations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brand/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9C985B2D-DEB4-AF45-8DFA-716EFBF2FF19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F36869-1AE6-434C-8C0A-C1DEFE4850BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="15620" xr2:uid="{BBF777D5-466C-F647-BCE9-E7DBB05CFFE3}"/>
   </bookViews>
@@ -34,49 +34,49 @@
     <t>name</t>
   </si>
   <si>
-    <t>EQU.ZA.STX500'</t>
-  </si>
-  <si>
     <t>STX500</t>
   </si>
   <si>
     <t>"Satrix S&amp;P 500 ETF"</t>
   </si>
   <si>
-    <t>EC10.EC.EC10'</t>
-  </si>
-  <si>
     <t>EC10</t>
   </si>
   <si>
     <t>"EasyCrypto 10"</t>
   </si>
   <si>
-    <t>EQU.ZA.NEWSLV'</t>
-  </si>
-  <si>
     <t>NEWSLV</t>
   </si>
   <si>
     <t>"New Wave Silver ETN"</t>
   </si>
   <si>
-    <t>EQU.ZA.NGPLT'</t>
-  </si>
-  <si>
     <t>NGPLT</t>
   </si>
   <si>
     <t>"NewPlat ETF"</t>
   </si>
   <si>
-    <t>EQU.ZA.STX40'</t>
-  </si>
-  <si>
     <t>STX40</t>
   </si>
   <si>
     <t>"Satrix 40 ETF"</t>
+  </si>
+  <si>
+    <t>EQU.ZA.STX500</t>
+  </si>
+  <si>
+    <t>EC10.EC.EC10</t>
+  </si>
+  <si>
+    <t>EQU.ZA.NEWSLV</t>
+  </si>
+  <si>
+    <t>EQU.ZA.NGPLT</t>
+  </si>
+  <si>
+    <t>EQU.ZA.STX40</t>
   </si>
 </sst>
 </file>
@@ -962,72 +962,72 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
       </c>
       <c r="C2">
         <v>0.2</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>0.2</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>0.2</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C5">
         <v>0.2</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C6">
         <v>0.2</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>